<commit_message>
Fase 168: Tipificación con los dos CDR de Wolkvox (v1.67.0)
- WhatsApp: HistChat por SKILL_ID (sin SKILL_NAME) reconocido como
  WhatsApp; nombre del skill desde el mapa por cliente (tabla
  skills_whatsapp, semilla ORLANT, GET/PUT /calidad/tipificacion/
  skills-whatsapp, editor solo admin en Cargar Datos). SKILL_ID 0 =
  salida; desconocidos se ignoran con un aviso agrupado.
- Llamadas: SKILL "-" = LLAMADAS DE SALIDA (no internalcall* ni sin tipo).
- Vista de ORLANT: Llamadas y WhatsApp lado a lado, sin tabla de detalle;
  tarjetas de salida solo en Llamadas (migración idempotente sobre la
  forma de la Fase 138; Mobilize no cambia).
- Plantillas, fichas y guía con la tabla de skills y la ruta pendiente
  de confirmar con Edwin.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/plantillas/PLANTILLA_TIPIFICACION_LLAMADAS.xlsx
+++ b/server/plantillas/PLANTILLA_TIPIFICACION_LLAMADAS.xlsx
@@ -476,7 +476,7 @@
         <v>De dónde sale</v>
       </c>
       <c r="B2" t="str">
-        <v>Wolkvox: Reportes → CDR → "1. Detalle de las llamadas", export completo (hoja "HistCDR&lt;fecha&gt;"). Se sube tal cual: el sistema nunca lee teléfonos, documentos ni comentarios.</v>
+        <v>Wolkvox: CDR de llamadas, export completo (hoja "HistCDR&lt;fecha&gt;") — [ruta pendiente de confirmar con Edwin]. Se sube tal cual: el sistema nunca lee teléfonos, documentos ni comentarios. SKILL_ID/SKILL_NAME "-" = Llamadas de salida (las internalcall no cuentan).</v>
       </c>
     </row>
     <row r="3">
@@ -621,7 +621,7 @@
         <v>Sí</v>
       </c>
       <c r="C14" t="str">
-        <v>Línea o skill (WhatsApp: "NOMBRE DE SKILL").</v>
+        <v>Línea o skill. "-" con TYPE_INTERACTION de salida = Llamadas de salida.</v>
       </c>
       <c r="D14" t="str">
         <v>SKILL SAC</v>

</xml_diff>

<commit_message>
Fase 174: reglas de ORLANT que confirmo Edwin (v1.71.0)
- out_pre es llamada de salida (outbound_ma, skill LLAMADAS DE SALIDA,
  SKILL_ID original conservado): no cuenta como entrada de CANCELACIONES.
- "No conectada" por cliente en el registro (salidaNoConectada):
  ORLANT NO_CONTESTAN + BUZON, MOBILIZE Cliente_no_contesta; migracion
  idempotente que no pisa cambios de un administrador.
- Plantillas de CDR con las 20 columnas del HistCDR y las 32 del HistChat.
- El lector acepta DATE como texto "aaaa-mm-dd hh:mm[:ss]".
- Pendientes, PROGRESS y bitacora; body-parser 2.4.0 (npm audit).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/plantillas/PLANTILLA_TIPIFICACION_LLAMADAS.xlsx
+++ b/server/plantillas/PLANTILLA_TIPIFICACION_LLAMADAS.xlsx
@@ -398,19 +398,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:T1"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
     <col min="3" max="3" width="14.83203125" customWidth="1"/>
     <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="21.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
     <col min="6" max="6" width="14.83203125" customWidth="1"/>
     <col min="7" max="7" width="14.83203125" customWidth="1"/>
     <col min="8" max="8" width="14.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="9" max="9" width="21.83203125" customWidth="1"/>
     <col min="10" max="10" width="14.83203125" customWidth="1"/>
-    <col min="11" max="11" width="14.83203125" customWidth="1"/>
+    <col min="11" max="11" width="23.83203125" customWidth="1"/>
+    <col min="12" max="12" width="18.83203125" customWidth="1"/>
+    <col min="13" max="13" width="14.83203125" customWidth="1"/>
+    <col min="14" max="14" width="14.83203125" customWidth="1"/>
+    <col min="15" max="15" width="14.83203125" customWidth="1"/>
+    <col min="16" max="16" width="14.83203125" customWidth="1"/>
+    <col min="17" max="17" width="14.83203125" customWidth="1"/>
+    <col min="18" max="18" width="14.83203125" customWidth="1"/>
+    <col min="19" max="19" width="14.83203125" customWidth="1"/>
+    <col min="20" max="20" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -421,43 +430,70 @@
         <v>DATE</v>
       </c>
       <c r="C1" t="str">
-        <v>HORA</v>
+        <v>DESTINY</v>
       </c>
       <c r="D1" t="str">
+        <v>TELEPHONE</v>
+      </c>
+      <c r="E1" t="str">
+        <v>COST</v>
+      </c>
+      <c r="F1" t="str">
+        <v>TIME_SEC</v>
+      </c>
+      <c r="G1" t="str">
         <v>TIME_MIN</v>
-      </c>
-      <c r="E1" t="str">
-        <v>DESCRIPTION_COD_ACT</v>
-      </c>
-      <c r="F1" t="str">
-        <v>SKILL_NAME</v>
-      </c>
-      <c r="G1" t="str">
-        <v>TIME_SEC</v>
       </c>
       <c r="H1" t="str">
         <v>COD_ACT</v>
       </c>
       <c r="I1" t="str">
+        <v>DESCRIPTION_COD_ACT</v>
+      </c>
+      <c r="J1" t="str">
+        <v>COD_ACT_2</v>
+      </c>
+      <c r="K1" t="str">
+        <v>DESCRIPTION_COD_ACT_2</v>
+      </c>
+      <c r="L1" t="str">
         <v>TYPE_INTERACTION</v>
       </c>
-      <c r="J1" t="str">
+      <c r="M1" t="str">
+        <v>CUSTOMER_ID</v>
+      </c>
+      <c r="N1" t="str">
         <v>HUNG_UP</v>
       </c>
-      <c r="K1" t="str">
+      <c r="O1" t="str">
+        <v>CAMPAIGN_ID</v>
+      </c>
+      <c r="P1" t="str">
+        <v>CONN_ID</v>
+      </c>
+      <c r="Q1" t="str">
         <v>SKILL_ID</v>
+      </c>
+      <c r="R1" t="str">
+        <v>SKILL_NAME</v>
+      </c>
+      <c r="S1" t="str">
+        <v>AGENT_ID</v>
+      </c>
+      <c r="T1" t="str">
+        <v>COMMENT</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E28"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -476,7 +512,7 @@
         <v>De dónde sale</v>
       </c>
       <c r="B2" t="str">
-        <v>Wolkvox: CDR de llamadas, export completo (hoja "HistCDR&lt;fecha&gt;") — [ruta pendiente de confirmar con Edwin]. Se sube tal cual: el sistema nunca lee teléfonos, documentos ni comentarios. SKILL_ID/SKILL_NAME "-" = Llamadas de salida (las internalcall no cuentan).</v>
+        <v>Wolkvox: CDR de llamadas, export completo (hoja "HistCDR&lt;fecha&gt;") — [ruta pendiente de confirmar con Edwin]. Se sube tal cual: el sistema nunca lee teléfonos, documentos ni comentarios. SKILL_ID/SKILL_NAME "-" = Llamadas de salida (las internalcall no cuentan). TYPE_INTERACTION "out_pre" también es Llamada de salida, aunque traiga skill (ORLANT: 4070 CANCELACIONES Y REPROGRAMACION).</v>
       </c>
     </row>
     <row r="3">
@@ -553,10 +589,10 @@
         <v>Sí</v>
       </c>
       <c r="C10" t="str">
-        <v>Fecha de la llamada (la hora va en HORA).</v>
+        <v>Fecha y hora de la llamada.</v>
       </c>
       <c r="D10" t="str">
-        <v>2026-08-01</v>
+        <v>2026-08-01 08:15:00</v>
       </c>
       <c r="E10" t="str">
         <v/>
@@ -564,16 +600,16 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>HORA</v>
+        <v>DESTINY</v>
       </c>
       <c r="B11" t="str">
         <v>No</v>
       </c>
       <c r="C11" t="str">
-        <v>Hora, si viene aparte.</v>
+        <v>Viene en el export de Wolkvox; el sistema nunca la lee ni la guarda.</v>
       </c>
       <c r="D11" t="str">
-        <v>08:15</v>
+        <v>3000000001</v>
       </c>
       <c r="E11" t="str">
         <v/>
@@ -581,16 +617,16 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>TIME_MIN</v>
+        <v>TELEPHONE</v>
       </c>
       <c r="B12" t="str">
         <v>No</v>
       </c>
       <c r="C12" t="str">
-        <v>Duración en minutos.</v>
-      </c>
-      <c r="D12">
-        <v>3</v>
+        <v>Viene en el export de Wolkvox; el sistema nunca la lee ni la guarda.</v>
+      </c>
+      <c r="D12" t="str">
+        <v>3000000001</v>
       </c>
       <c r="E12" t="str">
         <v/>
@@ -598,16 +634,16 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>DESCRIPTION_COD_ACT</v>
+        <v>COST</v>
       </c>
       <c r="B13" t="str">
-        <v>Sí</v>
+        <v>No</v>
       </c>
       <c r="C13" t="str">
-        <v>Motivo o tipificación.</v>
-      </c>
-      <c r="D13" t="str">
-        <v>Consulta general</v>
+        <v>Viene en el export de Wolkvox; el sistema no la usa.</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
       </c>
       <c r="E13" t="str">
         <v/>
@@ -615,33 +651,33 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>SKILL_NAME</v>
+        <v>TIME_SEC</v>
       </c>
       <c r="B14" t="str">
-        <v>Sí</v>
+        <v>No</v>
       </c>
       <c r="C14" t="str">
-        <v>Línea o skill. "-" con TYPE_INTERACTION de salida = Llamadas de salida.</v>
-      </c>
-      <c r="D14" t="str">
-        <v>SKILL SAC</v>
+        <v>Duración en segundos.</v>
+      </c>
+      <c r="D14">
+        <v>180</v>
       </c>
       <c r="E14" t="str">
-        <v>NOMBRE DE SKILL</v>
+        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>TIME_SEC</v>
+        <v>TIME_MIN</v>
       </c>
       <c r="B15" t="str">
         <v>No</v>
       </c>
       <c r="C15" t="str">
-        <v>Duración en segundos.</v>
+        <v>Duración en minutos.</v>
       </c>
       <c r="D15">
-        <v>180</v>
+        <v>3</v>
       </c>
       <c r="E15" t="str">
         <v/>
@@ -666,16 +702,16 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>TYPE_INTERACTION</v>
+        <v>DESCRIPTION_COD_ACT</v>
       </c>
       <c r="B17" t="str">
-        <v>No</v>
+        <v>Sí</v>
       </c>
       <c r="C17" t="str">
-        <v>"inbound" (entrante) u "outbound_ma" (saliente).</v>
+        <v>Motivo o tipificación. En una llamada de salida, el cliente define cuáles cuentan como "no conectada" (ORLANT: NO_CONTESTAN y BUZON).</v>
       </c>
       <c r="D17" t="str">
-        <v>inbound</v>
+        <v>Consulta general</v>
       </c>
       <c r="E17" t="str">
         <v/>
@@ -683,16 +719,16 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>HUNG_UP</v>
+        <v>COD_ACT_2</v>
       </c>
       <c r="B18" t="str">
         <v>No</v>
       </c>
       <c r="C18" t="str">
-        <v>Quién colgó ("agent" o "customer").</v>
+        <v>Viene en el export de Wolkvox; el sistema no la usa.</v>
       </c>
       <c r="D18" t="str">
-        <v>customer</v>
+        <v>-</v>
       </c>
       <c r="E18" t="str">
         <v/>
@@ -700,24 +736,177 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
+        <v>DESCRIPTION_COD_ACT_2</v>
+      </c>
+      <c r="B19" t="str">
+        <v>No</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Viene en el export de Wolkvox; el sistema no la usa.</v>
+      </c>
+      <c r="D19" t="str">
+        <v>-</v>
+      </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>TYPE_INTERACTION</v>
+      </c>
+      <c r="B20" t="str">
+        <v>No</v>
+      </c>
+      <c r="C20" t="str">
+        <v>"inbound" (entrante), "outbound_ma" u "out_pre" (salientes: las dos cuentan como Llamadas de salida). Las "internalcall" no cuentan como salida.</v>
+      </c>
+      <c r="D20" t="str">
+        <v>inbound</v>
+      </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>CUSTOMER_ID</v>
+      </c>
+      <c r="B21" t="str">
+        <v>No</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Viene en el export de Wolkvox; el sistema nunca la lee ni la guarda.</v>
+      </c>
+      <c r="D21" t="str">
+        <v>1000000001</v>
+      </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>HUNG_UP</v>
+      </c>
+      <c r="B22" t="str">
+        <v>No</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Quién colgó ("agent" o "customer").</v>
+      </c>
+      <c r="D22" t="str">
+        <v>customer</v>
+      </c>
+      <c r="E22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>CAMPAIGN_ID</v>
+      </c>
+      <c r="B23" t="str">
+        <v>No</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Viene en el export de Wolkvox; el sistema no la usa.</v>
+      </c>
+      <c r="D23" t="str">
+        <v>-</v>
+      </c>
+      <c r="E23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>CONN_ID</v>
+      </c>
+      <c r="B24" t="str">
+        <v>No</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Viene en el export de Wolkvox; el sistema nunca la lee ni la guarda.</v>
+      </c>
+      <c r="D24" t="str">
+        <v>EJEMPLO-0001</v>
+      </c>
+      <c r="E24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
         <v>SKILL_ID</v>
       </c>
-      <c r="B19" t="str">
-        <v>No</v>
-      </c>
-      <c r="C19" t="str">
+      <c r="B25" t="str">
+        <v>No</v>
+      </c>
+      <c r="C25" t="str">
         <v>Identificador técnico de la línea.</v>
       </c>
-      <c r="D19" t="str">
+      <c r="D25" t="str">
         <v>101</v>
       </c>
-      <c r="E19" t="str">
+      <c r="E25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>SKILL_NAME</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Sí</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Línea o skill. "-" con TYPE_INTERACTION de salida = Llamadas de salida.</v>
+      </c>
+      <c r="D26" t="str">
+        <v>SKILL SAC</v>
+      </c>
+      <c r="E26" t="str">
+        <v>NOMBRE DE SKILL</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>AGENT_ID</v>
+      </c>
+      <c r="B27" t="str">
+        <v>No</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Viene en el export de Wolkvox; el sistema nunca la lee ni la guarda.</v>
+      </c>
+      <c r="D27" t="str">
+        <v>0000</v>
+      </c>
+      <c r="E27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>COMMENT</v>
+      </c>
+      <c r="B28" t="str">
+        <v>No</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Viene en el export de Wolkvox; el sistema nunca la lee ni la guarda.</v>
+      </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
+      <c r="E28" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E28"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>